<commit_message>
docs: translate strategic workstream to Portuguese
</commit_message>
<xml_diff>
--- a/strategic-planning/payload/document/workstreams.xlsx
+++ b/strategic-planning/payload/document/workstreams.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorkStream" sheetId="1" r:id="Rd406c39aac184bb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorkStream" sheetId="1" r:id="R1566d15818e14a72"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -411,7 +411,7 @@
         </x:is>
       </x:c>
       <x:c r="B2" s="4" t="str">
-        <x:v>Strategic revenue workstream for the period from the September 2026 equinox to the September 2027 equinox, targeting R$250,000 in gross revenue. The plan is anchored by a primary PJ contract paying at least R$15,000 per month, ideally starting by October 2026 and no later than November 2026, with a desired duration of at least six months. Opportunities that depend centrally on Revit, Node.js, or React are excluded. Brasidata and InfoBIM are complementary revenue streams rather than immediate substitutes for the primary contract. Any new TechnipFMC engagement is counted only after a new contract is signed.</x:v>
+        <x:v>Planejamento estratégico para alcançar R$ 250 mil de receita bruta entre setembro de 2026 e setembro de 2027. O plano tem como base a obtenção de um contrato PJ principal, remoto, de pelo menos R$ 15 mil por mês, com início preferencial até outubro de 2026 — tolerando novembro — e duração mínima desejada de seis meses. A busca priorizará oportunidades com maior chance real de conversão e evitará posições centradas em Revit, Node.js ou React. As receitas da Brasidata e do InfoBIM serão complementares ao contrato principal. Um eventual novo trabalho com a TechnipFMC só será considerado após contrato efetivamente assinado.</x:v>
       </x:c>
       <x:c r="C2" s="4" t="inlineStr">
         <x:is>
@@ -419,7 +419,7 @@
         </x:is>
       </x:c>
       <x:c r="D2" s="4" t="str">
-        <x:v>Secure and maintain a primary PJ contract of at least R$15,000 per month and generate complementary revenue through Brasidata and InfoBIM to reach R$250,000 in gross revenue between September 2026 and September 2027.</x:v>
+        <x:v>Obter um contrato PJ principal de pelo menos R$ 15 mil por mês e gerar receitas complementares com a Brasidata e o InfoBIM, totalizando R$ 250 mil de receita bruta no período de setembro de 2026 a setembro de 2027.</x:v>
       </x:c>
       <x:c r="E2" s="3" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
docs: complete strategic workstream 5W2H
</commit_message>
<xml_diff>
--- a/strategic-planning/payload/document/workstreams.xlsx
+++ b/strategic-planning/payload/document/workstreams.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorkStream" sheetId="1" r:id="R1566d15818e14a72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorkStream" sheetId="1" r:id="R699689a8f2b44449"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -37,7 +37,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="5">
+  <x:cellXfs count="6">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -48,6 +48,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -344,12 +347,12 @@
     <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="58" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="42" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="42" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="58" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
@@ -373,38 +376,38 @@
           <x:t xml:space="preserve">What</x:t>
         </x:is>
       </x:c>
-      <x:c r="E1" s="1" t="inlineStr">
+      <x:c r="E1" s="5" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Why</x:t>
         </x:is>
       </x:c>
-      <x:c r="F1" s="1" t="inlineStr">
+      <x:c r="F1" s="5" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Who</x:t>
         </x:is>
       </x:c>
-      <x:c r="G1" s="1" t="inlineStr">
+      <x:c r="G1" s="5" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Where</x:t>
         </x:is>
       </x:c>
-      <x:c r="H1" s="1" t="inlineStr">
+      <x:c r="H1" s="5" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">When</x:t>
         </x:is>
       </x:c>
-      <x:c r="I1" s="1" t="inlineStr">
+      <x:c r="I1" s="5" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">How</x:t>
         </x:is>
       </x:c>
-      <x:c r="J1" s="1" t="inlineStr">
+      <x:c r="J1" s="5" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">HowMuch</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="2" ht="126" customHeight="1">
+    <x:row r="2" ht="250" customHeight="1">
       <x:c r="A2" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">b905b37c-f2d0-5c35-bed5-7190287d49b0</x:t>
@@ -421,35 +424,23 @@
       <x:c r="D2" s="4" t="str">
         <x:v>Obter um contrato PJ principal de pelo menos R$ 15 mil por mês e gerar receitas complementares com a Brasidata e o InfoBIM, totalizando R$ 250 mil de receita bruta no período de setembro de 2026 a setembro de 2027.</x:v>
       </x:c>
-      <x:c r="E2" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="F2" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="G2" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H2" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="I2" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="J2" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+      <x:c r="E2" s="4" t="str">
+        <x:v>Assegurar renda após o encerramento do contrato atual com a TechnipFMC e alcançar R$ 250 mil de receita bruta em doze meses, sem depender exclusivamente de um único contrato ou da conversão imediata da Brasidata e do InfoBIM.</x:v>
+      </x:c>
+      <x:c r="F2" s="4" t="str">
+        <x:v>Elias MP Junior, como responsável pela busca, seleção e conversão das oportunidades e pela execução comercial e técnica das receitas complementares da Brasidata e do InfoBIM.</x:v>
+      </x:c>
+      <x:c r="G2" s="4" t="str">
+        <x:v>Mercado brasileiro, priorizando contratos PJ remotos. Atuação presencial apenas quando fizer sentido para a contratação ou para a execução de serviços complementares.</x:v>
+      </x:c>
+      <x:c r="H2" s="4" t="str">
+        <x:v>Do equinócio de setembro de 2026 ao equinócio de setembro de 2027. O contrato principal deve começar preferencialmente até outubro de 2026, tolerando início em novembro, e ter duração mínima desejada de seis meses.</x:v>
+      </x:c>
+      <x:c r="I2" s="4" t="str">
+        <x:v>Preparar e operar uma pipeline de oportunidades no OntoBDC: capturar vagas e contatos, normalizar, validar, deduplicar, filtrar pelas restrições definidas, pontuar pela chance real de conversão e acompanhar cada oportunidade até contratação. Em paralelo, converter demandas reais em serviços da Brasidata e do InfoBIM.</x:v>
+      </x:c>
+      <x:c r="J2" s="4" t="str">
+        <x:v>Meta de R$ 250 mil de receita bruta no período. O contrato principal deve pagar no mínimo R$ 15 mil por mês; Brasidata e InfoBIM cobrem a parcela complementar necessária para atingir a meta.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>